<commit_message>
feat(vendor): make mobile optional and enforce strict GST validation
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/vendor-migration/vendor_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/vendor-migration/vendor_migration_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>name</t>
   </si>
@@ -32,7 +32,7 @@
     <t>Sector 17 Chandigarh</t>
   </si>
   <si>
-    <t>ABCD12345678EFZ</t>
+    <t>06ABCDE1234F1Z5</t>
   </si>
   <si>
     <t>9876543210</t>
@@ -44,10 +44,7 @@
     <t>Industrial Area Panchkula</t>
   </si>
   <si>
-    <t>PQRS87654321ZTA</t>
-  </si>
-  <si>
-    <t>9123456789</t>
+    <t>03PQRSX6789K2Z7</t>
   </si>
   <si>
     <t>Instructions</t>
@@ -56,10 +53,10 @@
     <t>Fill data in 'vendors' sheet only. Do not change header names.</t>
   </si>
   <si>
-    <t>Required columns: name, address, gst_no, mobile_no.</t>
-  </si>
-  <si>
-    <t>gst_no must be 15 chars (capital letters/digits). mobile_no must be 10 digits starting with 6-9.</t>
+    <t>Required columns: name, address, gst_no. mobile_no is optional.</t>
+  </si>
+  <si>
+    <t>gst_no format: 2 digits + 5 letters + 4 digits + 1 letter + 1 entity code (1-9/A-Z) + Z + 1 checksum (0-9/A-Z). Example: 06ABCDE1234F1Z5.</t>
   </si>
   <si>
     <t>This migration is insert-only. Existing gst_no or mobile_no will fail.</t>
@@ -487,9 +484,6 @@
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -507,27 +501,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(migration): make vendor GST optional in migration flow
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/vendor-migration/vendor_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/vendor-migration/vendor_migration_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>name</t>
   </si>
@@ -44,19 +44,16 @@
     <t>Industrial Area Panchkula</t>
   </si>
   <si>
-    <t>03PQRSX6789K2Z7</t>
-  </si>
-  <si>
     <t>Instructions</t>
   </si>
   <si>
     <t>Fill data in 'vendors' sheet only. Do not change header names.</t>
   </si>
   <si>
-    <t>Required columns: name, address, gst_no. mobile_no is optional.</t>
-  </si>
-  <si>
-    <t>gst_no format: 2 digits + 5 letters + 4 digits + 1 letter + 1 entity code (1-9/A-Z) + Z + 1 checksum (0-9/A-Z). Example: 06ABCDE1234F1Z5.</t>
+    <t>Required columns: name, address. gst_no and mobile_no are optional.</t>
+  </si>
+  <si>
+    <t>If provided, gst_no format: 2 digits + 5 letters + 4 digits + 1 letter + 1 entity code (1-9/A-Z) + Z + 1 checksum (0-9/A-Z). Example: 06ABCDE1234F1Z5.</t>
   </si>
   <si>
     <t>This migration is insert-only. Existing gst_no or mobile_no will fail.</t>
@@ -481,9 +478,6 @@
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -501,27 +495,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(vendor): support practical vendor names in API and migration
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/vendor-migration/vendor_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/vendor-migration/vendor_migration_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>name</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Required columns: name, address. gst_no and mobile_no are optional.</t>
+  </si>
+  <si>
+    <t>name can include letters, numbers, spaces, and symbols (&amp; . , ' ( ) / -). Multiple spaces are normalized automatically.</t>
   </si>
   <si>
     <t>If provided, gst_no format: 2 digits + 5 letters + 4 digits + 1 letter + 1 entity code (1-9/A-Z) + Z + 1 checksum (0-9/A-Z). Example: 06ABCDE1234F1Z5.</t>
@@ -487,7 +490,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
@@ -518,6 +521,11 @@
         <v>14</v>
       </c>
     </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>